<commit_message>
fix: sanitize excel typos, implement smart tag matching in worker, and render choices in wrong notes
</commit_message>
<xml_diff>
--- a/excels/1급_전산회계책_필기.xlsx
+++ b/excels/1급_전산회계책_필기.xlsx
@@ -1637,7 +1637,7 @@
       <c r="C30" t="inlineStr">
         <is>
           <t>주 식 취득시
-(차) 단기매매증권 2,000,000원 (대) 현통예금 2,000,000원</t>
+(차) 단기매매증권 2,000,000원 (대) 보통예금 2,000,000원</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1649,7 +1649,7 @@
       <c r="E30" t="inlineStr">
         <is>
           <t>제 2기 1월 1일
-(차) 현통예금 1,500,000원 (대) 단 기매매증권 1,000,000원
+(차) 보통예금 1,500,000원 (대) 단기매매증권 1,000,000원
 단기매매증권처분이익 500,000원</t>
         </is>
       </c>
@@ -1891,7 +1891,7 @@
       <c r="C36" t="inlineStr">
         <is>
           <t>주 식 취득시
-(차) 단기매매증권 2,000,000원 (대) 현통예금 2,000,000원</t>
+(차) 단기매매증권 2,000,000원 (대) 보통예금 2,000,000원</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1903,7 +1903,7 @@
       <c r="E36" t="inlineStr">
         <is>
           <t>제 2기 1월 1일
-(차) 현통예금 1,500,000원 (대) 단 기매매증권 1,000,000원
+(차) 보통예금 1,500,000원 (대) 단기매매증권 1,000,000원
 단기매매증권처분이익 500,000원</t>
         </is>
       </c>
@@ -16064,7 +16064,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>처분이익 : (50주 × 25,000원 (장부가액)) - (50주 × 30,000원 (처분가액)) = 250,000 원 (차) 현금 1,500,000원 (대) 단 기매매증권 1,250,000원 단기매매증권처분이익 250,000원 A사 주식 단기매매증권평가이익 100,000원 + 배당금수익 60,000원 = 160,000원</t>
+          <t>처분이익 : (50주 × 25,000원 (장부가액)) - (50주 × 30,000원 (처분가액)) = 250,000 원 (차) 현금 1,500,000원 (대) 단기매매증권 1,250,000원 단기매매증권처분이익 250,000원 A사 주식 단기매매증권평가이익 100,000원 + 배당금수익 60,000원 = 160,000원</t>
         </is>
       </c>
     </row>
@@ -16424,7 +16424,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>처분이익 : (50주 × 25,000원 (장부가액)) - (50주 × 30,000원 (처분가액)) = 250,000 원 (차) 현금 1,500,000원 (대) 단 기매매증권 1,250,000원 단기매매증권처분이익 250,000원 A사 주식 단기매매증권평가이익 100,000원 + 배당금수익 60,000원 = 160,000원</t>
+          <t>처분이익 : (50주 × 25,000원 (장부가액)) - (50주 × 30,000원 (처분가액)) = 250,000 원 (차) 현금 1,500,000원 (대) 단기매매증권 1,250,000원 단기매매증권처분이익 250,000원 A사 주식 단기매매증권평가이익 100,000원 + 배당금수익 60,000원 = 160,000원</t>
         </is>
       </c>
     </row>
@@ -16509,12 +16509,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>개별법은 재고자산의 단가결정방법이다.</t>
+          <t>처분이익 = (50주 × 30,000원 (처분가액)) - (50주 × 25,000원 (장부가액)) = 250,000원. 올바른 분개: (차) 보통예금 1,500,000원 / (대) 단기매매증권 1,250,000원, 단기매매증권처분이익 250,000원 (보기 3번은 취득원가 20,000원을 기준으로 장부가 100만원을 제거하고 처분이익 50만원을 계상하여 틀렸습니다.)</t>
         </is>
       </c>
     </row>

</xml_diff>